<commit_message>
Lab8: HashSet вместо List.Contains (этап 2)
</commit_message>
<xml_diff>
--- a/Lab8/Lab8/Лист Microsoft Excel.xlsx
+++ b/Lab8/Lab8/Лист Microsoft Excel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\123\tp-labs-Petuhova\Lab8\Lab8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0E14A7-844A-42EF-8A97-8D83631339D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7949A563-530C-4AC8-B807-3371328D5297}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6732" yWindow="1176" windowWidth="22692" windowHeight="11496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13620" yWindow="5052" windowWidth="22692" windowHeight="11496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -469,7 +469,9 @@
       <c r="B2" s="7">
         <v>483</v>
       </c>
-      <c r="C2" s="7"/>
+      <c r="C2" s="7">
+        <v>2</v>
+      </c>
       <c r="D2" s="7"/>
       <c r="E2" s="4"/>
     </row>
@@ -480,7 +482,9 @@
       <c r="B3" s="8">
         <v>3284</v>
       </c>
-      <c r="C3" s="8"/>
+      <c r="C3" s="8">
+        <v>3255</v>
+      </c>
       <c r="D3" s="8"/>
       <c r="E3" s="4"/>
     </row>
@@ -491,7 +495,9 @@
       <c r="B4" s="8">
         <v>1465</v>
       </c>
-      <c r="C4" s="8"/>
+      <c r="C4" s="8">
+        <v>1395</v>
+      </c>
       <c r="D4" s="8"/>
       <c r="E4" s="4"/>
     </row>
@@ -502,7 +508,9 @@
       <c r="B5" s="8">
         <v>1090</v>
       </c>
-      <c r="C5" s="7"/>
+      <c r="C5" s="7">
+        <v>1195</v>
+      </c>
       <c r="D5" s="7"/>
       <c r="E5" s="4"/>
     </row>
@@ -514,7 +522,9 @@
         <f>SUM(B2:B5)</f>
         <v>6322</v>
       </c>
-      <c r="C6" s="7"/>
+      <c r="C6" s="7">
+        <v>5893</v>
+      </c>
       <c r="D6" s="7"/>
       <c r="E6" s="4"/>
     </row>

</xml_diff>